<commit_message>
added finetune shell file for diffusion prior
</commit_message>
<xml_diff>
--- a/ExperimentData.xlsx
+++ b/ExperimentData.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zhc/Documents/PhD/projects/ImagenFew/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94F170E5-789B-2640-814A-ECABDFFA2EBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DD90CED-2F28-2349-8930-BCEF1A179FB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6220" yWindow="2640" windowWidth="31320" windowHeight="13060" xr2:uid="{E5419BAC-4B6F-E540-9397-DA349BE39778}"/>
+    <workbookView xWindow="17740" yWindow="2600" windowWidth="31420" windowHeight="13060" xr2:uid="{E5419BAC-4B6F-E540-9397-DA349BE39778}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="27">
   <si>
     <t>ETTh2</t>
   </si>
@@ -81,6 +81,42 @@
   </si>
   <si>
     <t>Mine</t>
+  </si>
+  <si>
+    <t>Neurip2025</t>
+  </si>
+  <si>
+    <t>Neurips2024</t>
+  </si>
+  <si>
+    <t>old</t>
+  </si>
+  <si>
+    <t>Weather</t>
+  </si>
+  <si>
+    <t>StarLightCurves</t>
+  </si>
+  <si>
+    <t>Sine</t>
+  </si>
+  <si>
+    <t>SelfRegulationSCP1</t>
+  </si>
+  <si>
+    <t>SaugeenRiverFlow</t>
+  </si>
+  <si>
+    <t>ILI</t>
+  </si>
+  <si>
+    <t>ETThm1</t>
+  </si>
+  <si>
+    <t>ETThm2</t>
+  </si>
+  <si>
+    <t>Avg</t>
   </si>
 </sst>
 </file>
@@ -118,12 +154,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="5" tint="0.59999389629810485"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="9" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -131,6 +161,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="8" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -147,7 +183,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -155,24 +191,28 @@
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -507,11 +547,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EFA88CAE-8538-1C4B-BF78-B0AFB8480CBE}">
-  <dimension ref="E7:M16"/>
+  <dimension ref="E7:M34"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="5" max="5" width="12.6640625" customWidth="1"/>
-    <col min="10" max="10" width="16.83203125" customWidth="1"/>
+    <col min="6" max="6" width="19.33203125" customWidth="1"/>
+    <col min="10" max="10" width="18.1640625" customWidth="1"/>
     <col min="11" max="11" width="17.6640625" customWidth="1"/>
     <col min="12" max="12" width="15.5" customWidth="1"/>
     <col min="13" max="13" width="15.6640625" customWidth="1"/>
@@ -520,11 +561,11 @@
     <row r="7" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E7" s="1"/>
       <c r="F7" s="1"/>
-      <c r="G7" s="3" t="s">
+      <c r="G7" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
       <c r="J7" s="2" t="s">
         <v>14</v>
       </c>
@@ -535,57 +576,63 @@
     <row r="8" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E8" s="1"/>
       <c r="F8" s="1"/>
-      <c r="G8" s="5"/>
-      <c r="H8" s="5"/>
-      <c r="I8" s="5"/>
-      <c r="J8" s="8"/>
-      <c r="K8" s="4" t="s">
+      <c r="G8" s="8"/>
+      <c r="H8" s="8"/>
+      <c r="I8" s="8"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="L8" s="4"/>
-      <c r="M8" s="4"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
     </row>
     <row r="9" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E9" s="1"/>
       <c r="F9" s="1"/>
-      <c r="G9" s="5"/>
-      <c r="H9" s="5"/>
-      <c r="I9" s="5"/>
-      <c r="J9" s="8" t="s">
+      <c r="G9" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="H9" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="J9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="K9" s="7" t="s">
+      <c r="K9" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="L9" s="7" t="s">
+      <c r="L9" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="M9" s="7" t="s">
+      <c r="M9" s="5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E10" s="1"/>
       <c r="F10" s="1"/>
-      <c r="G10" s="5" t="s">
+      <c r="G10" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="H10" s="5" t="s">
+      <c r="H10" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="J10" s="8" t="s">
+      <c r="J10" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="K10" s="7" t="s">
+      <c r="K10" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="L10" s="7" t="s">
+      <c r="L10" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="M10" s="7" t="s">
+      <c r="M10" s="5" t="s">
         <v>11</v>
       </c>
     </row>
@@ -596,128 +643,386 @@
       <c r="F11" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G11" s="5">
+      <c r="G11" s="8">
         <v>5.6000000000000001E-2</v>
       </c>
-      <c r="H11" s="5">
+      <c r="H11" s="8">
         <v>0.151</v>
       </c>
-      <c r="I11" s="5">
+      <c r="I11" s="8">
         <v>1.804</v>
       </c>
-      <c r="J11" s="6">
+      <c r="J11" s="4">
         <v>2.7E-2</v>
       </c>
-      <c r="K11" s="7"/>
-      <c r="L11" s="7"/>
-      <c r="M11" s="7"/>
+      <c r="K11" s="5"/>
+      <c r="L11" s="5"/>
+      <c r="M11" s="5"/>
     </row>
     <row r="12" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E12" s="1"/>
       <c r="F12" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G12" s="5">
+      <c r="G12" s="8">
         <v>3.6999999999999998E-2</v>
       </c>
-      <c r="H12" s="5">
+      <c r="H12" s="8">
         <v>1.056</v>
       </c>
-      <c r="I12" s="5">
+      <c r="I12" s="8">
         <v>0.248</v>
       </c>
-      <c r="J12" s="6">
+      <c r="J12" s="4">
         <v>0.02</v>
       </c>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
+      <c r="K12" s="5"/>
+      <c r="L12" s="5"/>
+      <c r="M12" s="5"/>
     </row>
     <row r="13" spans="5:13" x14ac:dyDescent="0.2">
       <c r="E13" s="1"/>
       <c r="F13" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G13" s="5">
+      <c r="G13" s="8">
         <v>0.249</v>
       </c>
-      <c r="H13" s="5">
+      <c r="H13" s="8">
         <v>0.26</v>
       </c>
-      <c r="I13" s="5">
+      <c r="I13" s="8">
         <v>0.307</v>
       </c>
-      <c r="J13" s="6">
+      <c r="J13" s="4">
         <v>7.0000000000000007E-2</v>
       </c>
-      <c r="K13" s="7"/>
-      <c r="L13" s="7"/>
-      <c r="M13" s="7"/>
+      <c r="K13" s="5"/>
+      <c r="L13" s="5"/>
+      <c r="M13" s="5"/>
     </row>
     <row r="14" spans="5:13" x14ac:dyDescent="0.2">
-      <c r="E14" s="1" t="s">
+      <c r="F14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G14" s="8">
+        <v>1.4590000000000001</v>
+      </c>
+      <c r="H14" s="8">
+        <v>2.2467999999999999</v>
+      </c>
+      <c r="I14" s="8">
+        <v>5.2359999999999998</v>
+      </c>
+    </row>
+    <row r="15" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F15" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" s="8">
+        <v>1.0500000000000001E-2</v>
+      </c>
+      <c r="H15" s="8">
+        <v>8.2000000000000007E-3</v>
+      </c>
+      <c r="I15" s="8">
+        <v>7.9000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="16" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F16" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G16" s="8">
+        <v>3.15E-3</v>
+      </c>
+      <c r="H16" s="8">
+        <v>1.6899999999999998E-2</v>
+      </c>
+      <c r="I16" s="8">
+        <v>1.1900000000000001E-2</v>
+      </c>
+    </row>
+    <row r="17" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F17" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G17" s="8">
+        <v>2.17</v>
+      </c>
+      <c r="H17" s="8">
+        <v>1.4490000000000001</v>
+      </c>
+      <c r="I17" s="8">
+        <v>1.861</v>
+      </c>
+    </row>
+    <row r="18" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F18" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G18" s="8">
+        <v>8.5000000000000006E-3</v>
+      </c>
+      <c r="H18" s="8">
+        <v>4.6699999999999997E-3</v>
+      </c>
+      <c r="I18" s="8">
+        <v>1.02</v>
+      </c>
+    </row>
+    <row r="19" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F19" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G19" s="8">
+        <v>1.5329999999999999</v>
+      </c>
+      <c r="H19" s="8">
+        <v>1.921</v>
+      </c>
+      <c r="I19" s="8">
+        <v>1.718</v>
+      </c>
+    </row>
+    <row r="20" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F20" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G20" s="8">
+        <v>8.3199999999999993E-3</v>
+      </c>
+      <c r="H20" s="8">
+        <v>1.49E-2</v>
+      </c>
+      <c r="I20" s="8">
+        <v>1.9890000000000001</v>
+      </c>
+    </row>
+    <row r="21" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F21" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G21" s="8">
+        <v>2.4E-2</v>
+      </c>
+      <c r="H21" s="8">
+        <v>3.3700000000000001E-2</v>
+      </c>
+      <c r="I21" s="8">
+        <v>1.6319999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F22" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="G22" s="10">
+        <f>AVERAGE(G11:G21)</f>
+        <v>0.50531545454545457</v>
+      </c>
+      <c r="H22" s="10">
+        <f t="shared" ref="H22:I22" si="0">AVERAGE(H11:H21)</f>
+        <v>0.65110636363636365</v>
+      </c>
+      <c r="I22" s="10">
+        <f t="shared" si="0"/>
+        <v>1.4459909090909091</v>
+      </c>
+    </row>
+    <row r="23" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E23" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="F14" s="1" t="s">
+      <c r="F23" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G14" s="5">
+      <c r="G23" s="8">
         <v>1.0999999999999999E-2</v>
       </c>
-      <c r="H14" s="5">
+      <c r="H23" s="8">
         <v>3.3000000000000002E-2</v>
       </c>
-      <c r="I14" s="5">
+      <c r="I23" s="8">
         <v>0.28000000000000003</v>
       </c>
-      <c r="J14" s="6">
+      <c r="J23" s="4">
         <v>6.0000000000000001E-3</v>
       </c>
-      <c r="K14" s="7"/>
-      <c r="L14" s="7"/>
-      <c r="M14" s="7"/>
-    </row>
-    <row r="15" spans="5:13" x14ac:dyDescent="0.2">
-      <c r="E15" s="1"/>
-      <c r="F15" s="1" t="s">
+      <c r="K23" s="5"/>
+      <c r="L23" s="5"/>
+      <c r="M23" s="5"/>
+    </row>
+    <row r="24" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E24" s="1"/>
+      <c r="F24" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G15" s="5">
+      <c r="G24" s="8">
         <v>1.4E-2</v>
       </c>
-      <c r="H15" s="5">
+      <c r="H24" s="8">
         <v>0.28899999999999998</v>
       </c>
-      <c r="I15" s="5">
+      <c r="I24" s="8">
         <v>9.2999999999999999E-2</v>
       </c>
-      <c r="J15" s="6">
+      <c r="J24" s="4">
         <v>1.2E-2</v>
       </c>
-      <c r="K15" s="7"/>
-      <c r="L15" s="7"/>
-      <c r="M15" s="7"/>
-    </row>
-    <row r="16" spans="5:13" x14ac:dyDescent="0.2">
-      <c r="E16" s="1"/>
-      <c r="F16" s="1" t="s">
+      <c r="K24" s="5"/>
+      <c r="L24" s="5"/>
+      <c r="M24" s="5"/>
+    </row>
+    <row r="25" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="E25" s="1"/>
+      <c r="F25" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G16" s="5">
+      <c r="G25" s="8">
         <v>3.9E-2</v>
       </c>
-      <c r="H16" s="5">
+      <c r="H25" s="8">
         <v>7.0999999999999994E-2</v>
       </c>
-      <c r="I16" s="5">
+      <c r="I25" s="8">
         <v>0.11</v>
       </c>
-      <c r="J16" s="6">
+      <c r="J25" s="4">
         <v>1.6E-2</v>
       </c>
-      <c r="K16" s="7"/>
-      <c r="L16" s="7"/>
-      <c r="M16" s="7"/>
+      <c r="K25" s="5"/>
+      <c r="L25" s="5"/>
+      <c r="M25" s="5"/>
+    </row>
+    <row r="26" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F26" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="G26" s="8">
+        <v>0.1986</v>
+      </c>
+      <c r="H26" s="8">
+        <v>1.9300000000000001E-2</v>
+      </c>
+      <c r="I26" s="8">
+        <v>0.4138</v>
+      </c>
+    </row>
+    <row r="27" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="G27" s="8">
+        <v>1.0699999999999999E-2</v>
+      </c>
+      <c r="H27" s="8">
+        <v>1.37E-2</v>
+      </c>
+      <c r="I27" s="8">
+        <v>3.1699999999999999E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F28" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="G28" s="8">
+        <v>9.5999999999999992E-3</v>
+      </c>
+      <c r="H28" s="8">
+        <v>1.0699999999999999E-2</v>
+      </c>
+      <c r="I28" s="8">
+        <v>2.5000000000000001E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F29" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="G29" s="8">
+        <v>0.45500000000000002</v>
+      </c>
+      <c r="H29" s="10">
+        <v>0.28299999999999997</v>
+      </c>
+      <c r="I29" s="8">
+        <v>0.16389999999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F30" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G30" s="8">
+        <v>5.1000000000000004E-3</v>
+      </c>
+      <c r="H30" s="10">
+        <v>4.7999999999999996E-3</v>
+      </c>
+      <c r="I30" s="8">
+        <v>0.1067</v>
+      </c>
+    </row>
+    <row r="31" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F31" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="G31" s="8">
+        <v>0.38629999999999998</v>
+      </c>
+      <c r="H31" s="10">
+        <v>0.42380000000000001</v>
+      </c>
+      <c r="I31" s="8">
+        <v>0.379</v>
+      </c>
+    </row>
+    <row r="32" spans="5:13" x14ac:dyDescent="0.2">
+      <c r="F32" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="G32" s="8">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="H32" s="8">
+        <v>6.4999999999999997E-3</v>
+      </c>
+      <c r="I32" s="8">
+        <v>0.31459999999999999</v>
+      </c>
+    </row>
+    <row r="33" spans="6:9" x14ac:dyDescent="0.2">
+      <c r="F33" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="G33" s="8">
+        <v>6.0000000000000001E-3</v>
+      </c>
+      <c r="H33" s="8">
+        <v>9.1999999999999998E-3</v>
+      </c>
+      <c r="I33" s="8">
+        <v>0.22670000000000001</v>
+      </c>
+    </row>
+    <row r="34" spans="6:9" x14ac:dyDescent="0.2">
+      <c r="F34" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="G34" s="10">
+        <f>AVERAGE(G24:G33,G23)</f>
+        <v>0.10349090909090909</v>
+      </c>
+      <c r="H34" s="10">
+        <f t="shared" ref="H34:I34" si="1">AVERAGE(H24:H33,H23)</f>
+        <v>0.10581818181818181</v>
+      </c>
+      <c r="I34" s="10">
+        <f t="shared" si="1"/>
+        <v>0.19494545454545456</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>